<commit_message>
feat: add SHAP analysis scripts, visualization plots, and feature importance rankings for multiple models
</commit_message>
<xml_diff>
--- a/olah/model_2_MSC_var_Oke/olah/4. SHAP/shap_importance_3model.xlsx
+++ b/olah/model_2_MSC_var_Oke/olah/4. SHAP/shap_importance_3model.xlsx
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.04655353269630365</v>
+        <v>0.0463468381800551</v>
       </c>
       <c r="C2" t="n">
         <v>0.3051705358256179</v>
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.08419119551156057</v>
+        <v>0.08422997421689241</v>
       </c>
       <c r="C3" t="n">
         <v>0.5038448546869752</v>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02592063502769194</v>
+        <v>0.02589038545411225</v>
       </c>
       <c r="C4" t="n">
         <v>0.153851668354746</v>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02028880002992595</v>
+        <v>0.02048546915584849</v>
       </c>
       <c r="C5" t="n">
         <v>0.4954960818544649</v>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.03356006614718429</v>
+        <v>0.03361090533621575</v>
       </c>
       <c r="C6" t="n">
         <v>0.2587262901187525</v>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.03695709740328559</v>
+        <v>0.03689732544436627</v>
       </c>
       <c r="C7" t="n">
         <v>0.1500998572606453</v>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.02470075572112229</v>
+        <v>0.02495262520288738</v>
       </c>
       <c r="C8" t="n">
         <v>0.2873532725110888</v>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02358757085671901</v>
+        <v>0.02359549713688154</v>
       </c>
       <c r="C9" t="n">
         <v>0.2540568703687955</v>

</xml_diff>